<commit_message>
Add a VMTW co-chair and host to session 1
Session 1, Medical Imaging and Diagnostic Deep Learning, opens the technical programme
on Monday at 11:00 and still had no joining link. D. Geetha, a VMTW standby volunteer
who is free at that time, joins as co-chair and hosts the meeting with their own Meet
link. Prof. Diwakar Shukla remains chair and joins through it. The session 1 chair
sheet is regenerated with the link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/programme/chair-sheets/S01.xlsx
+++ b/programme/chair-sheets/S01.xlsx
@@ -52,13 +52,13 @@
     <t xml:space="preserve">Co-chair</t>
   </si>
   <si>
-    <t xml:space="preserve">-</t>
+    <t xml:space="preserve">D. Geetha</t>
   </si>
   <si>
     <t xml:space="preserve">Joining link</t>
   </si>
   <si>
-    <t xml:space="preserve">to be confirmed</t>
+    <t xml:space="preserve">https://meet.google.com/pqz-zpbv-htc</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>

</xml_diff>